<commit_message>
corpus(rs2 joints): every workbook carries the initial stress its row is solved with
The rows without a strength-reduction tag (RJ-3, RJ-5, RJ-6, RJ-20) and the
tilt row RJ-16 were written with no K0, and the figure producer supplied
k0 = 1 from its own table, so the workbook alone did not reproduce the row.
The producer's row tables move to rs2_joint_cases.py, shared with the
builder, and the builder writes the K0 a row's tag or table entry names.
The five workbooks differ from before in one cell each (main!D16).

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/verification/files/rocscience/joints/rj003.xlsx
+++ b/docs/verification/files/rocscience/joints/rj003.xlsx
@@ -3374,7 +3374,9 @@
       <c r="G16" t="s">
         <v>34</v>
       </c>
-      <c r="D16"/>
+      <c r="D16">
+        <v>1.0</v>
+      </c>
     </row>
     <row r="17" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B17" s="1"/>

</xml_diff>

<commit_message>
verification(rs2 joints): the four Lorig & Varona rows are posed on the vendor's file again; the chapter's printed list and the cohesion-only reading stay beside as notes
Norm's ruling of 2026-09-30 evening. The chapter prints one property list for
the section (joints friction only, a rock that can yield) and never says the
list was used unchanged in its toppling runs; taken literally it reproduces the
chapter's answer only on problem 7 and on problem 5 neither its answer nor its
mechanism (the slabs slide on the face-parallel joints and the toe rock yields,
1.096 against UDEC 1.70). The rows therefore return to the vendor's file (RJ-3
1.232 red, RJ-4 1.311 green, RJ-5 1.857 red, RJ-7 1.564 yellow), with the
chapter-list runs kept as rj00X_chapter workbooks and tagged notes, and the
cohesion-only diagnostic as a one-line note allowed by ruling.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/verification/files/rocscience/joints/rj003.xlsx
+++ b/docs/verification/files/rocscience/joints/rj003.xlsx
@@ -4939,7 +4939,9 @@
       <c r="F3" s="3">
         <v>51.9993775139</v>
       </c>
-      <c r="G3" s="3"/>
+      <c r="G3" s="3">
+        <v>100.0</v>
+      </c>
       <c r="H3" s="3">
         <v>40.0</v>
       </c>
@@ -4976,7 +4978,9 @@
       <c r="F4" s="3">
         <v>110.4754655171</v>
       </c>
-      <c r="G4" s="3"/>
+      <c r="G4" s="3">
+        <v>100.0</v>
+      </c>
       <c r="H4" s="3">
         <v>40.0</v>
       </c>
@@ -5013,7 +5017,9 @@
       <c r="F5" s="3">
         <v>140.0</v>
       </c>
-      <c r="G5" s="3"/>
+      <c r="G5" s="3">
+        <v>100.0</v>
+      </c>
       <c r="H5" s="3">
         <v>40.0</v>
       </c>
@@ -5050,7 +5056,9 @@
       <c r="F6" s="3">
         <v>140.0</v>
       </c>
-      <c r="G6" s="3"/>
+      <c r="G6" s="3">
+        <v>100.0</v>
+      </c>
       <c r="H6" s="3">
         <v>40.0</v>
       </c>
@@ -5087,7 +5095,9 @@
       <c r="F7" s="3">
         <v>140.0</v>
       </c>
-      <c r="G7" s="3"/>
+      <c r="G7" s="3">
+        <v>100.0</v>
+      </c>
       <c r="H7" s="3">
         <v>40.0</v>
       </c>
@@ -5124,7 +5134,9 @@
       <c r="F8" s="3">
         <v>140.0</v>
       </c>
-      <c r="G8" s="3"/>
+      <c r="G8" s="3">
+        <v>100.0</v>
+      </c>
       <c r="H8" s="3">
         <v>40.0</v>
       </c>
@@ -5161,7 +5173,9 @@
       <c r="F9" s="3">
         <v>140.0</v>
       </c>
-      <c r="G9" s="3"/>
+      <c r="G9" s="3">
+        <v>100.0</v>
+      </c>
       <c r="H9" s="3">
         <v>40.0</v>
       </c>
@@ -5198,7 +5212,9 @@
       <c r="F10" s="3">
         <v>140.0</v>
       </c>
-      <c r="G10" s="3"/>
+      <c r="G10" s="3">
+        <v>100.0</v>
+      </c>
       <c r="H10" s="3">
         <v>40.0</v>
       </c>
@@ -5235,7 +5251,9 @@
       <c r="F11" s="3">
         <v>140.0</v>
       </c>
-      <c r="G11" s="3"/>
+      <c r="G11" s="3">
+        <v>100.0</v>
+      </c>
       <c r="H11" s="3">
         <v>40.0</v>
       </c>
@@ -5272,7 +5290,9 @@
       <c r="F12" s="3">
         <v>158.3344152734</v>
       </c>
-      <c r="G12" s="3"/>
+      <c r="G12" s="3">
+        <v>100.0</v>
+      </c>
       <c r="H12" s="3">
         <v>40.0</v>
       </c>
@@ -5309,7 +5329,9 @@
       <c r="F13" s="3">
         <v>178.322823806</v>
       </c>
-      <c r="G13" s="3"/>
+      <c r="G13" s="3">
+        <v>100.0</v>
+      </c>
       <c r="H13" s="3">
         <v>40.0</v>
       </c>
@@ -5346,7 +5368,9 @@
       <c r="F14" s="3">
         <v>198.3112323386</v>
       </c>
-      <c r="G14" s="3"/>
+      <c r="G14" s="3">
+        <v>100.0</v>
+      </c>
       <c r="H14" s="3">
         <v>40.0</v>
       </c>
@@ -5383,7 +5407,9 @@
       <c r="F15" s="3">
         <v>218.2996408711</v>
       </c>
-      <c r="G15" s="3"/>
+      <c r="G15" s="3">
+        <v>100.0</v>
+      </c>
       <c r="H15" s="3">
         <v>40.0</v>
       </c>
@@ -5420,7 +5446,9 @@
       <c r="F16" s="3">
         <v>238.2880494037</v>
       </c>
-      <c r="G16" s="3"/>
+      <c r="G16" s="3">
+        <v>100.0</v>
+      </c>
       <c r="H16" s="3">
         <v>40.0</v>
       </c>
@@ -5457,7 +5485,9 @@
       <c r="F17" s="3">
         <v>258.2764579362</v>
       </c>
-      <c r="G17" s="3"/>
+      <c r="G17" s="3">
+        <v>100.0</v>
+      </c>
       <c r="H17" s="3">
         <v>40.0</v>
       </c>
@@ -5494,7 +5524,9 @@
       <c r="F18" s="3">
         <v>278.2648664688</v>
       </c>
-      <c r="G18" s="3"/>
+      <c r="G18" s="3">
+        <v>100.0</v>
+      </c>
       <c r="H18" s="3">
         <v>40.0</v>
       </c>
@@ -5531,7 +5563,9 @@
       <c r="F19" s="3">
         <v>298.2532750014</v>
       </c>
-      <c r="G19" s="3"/>
+      <c r="G19" s="3">
+        <v>100.0</v>
+      </c>
       <c r="H19" s="3">
         <v>40.0</v>
       </c>
@@ -5568,7 +5602,9 @@
       <c r="F20" s="3">
         <v>318.2416835339</v>
       </c>
-      <c r="G20" s="3"/>
+      <c r="G20" s="3">
+        <v>100.0</v>
+      </c>
       <c r="H20" s="3">
         <v>40.0</v>
       </c>
@@ -5605,7 +5641,9 @@
       <c r="F21" s="3">
         <v>338.2300920665</v>
       </c>
-      <c r="G21" s="3"/>
+      <c r="G21" s="3">
+        <v>100.0</v>
+      </c>
       <c r="H21" s="3">
         <v>40.0</v>
       </c>
@@ -5642,7 +5680,9 @@
       <c r="F22" s="3">
         <v>358.2185005991</v>
       </c>
-      <c r="G22" s="3"/>
+      <c r="G22" s="3">
+        <v>100.0</v>
+      </c>
       <c r="H22" s="3">
         <v>40.0</v>
       </c>
@@ -5679,7 +5719,9 @@
       <c r="F23" s="3">
         <v>378.2069091316</v>
       </c>
-      <c r="G23" s="3"/>
+      <c r="G23" s="3">
+        <v>100.0</v>
+      </c>
       <c r="H23" s="3">
         <v>40.0</v>
       </c>
@@ -5716,7 +5758,9 @@
       <c r="F24" s="3">
         <v>398.1953176642</v>
       </c>
-      <c r="G24" s="3"/>
+      <c r="G24" s="3">
+        <v>100.0</v>
+      </c>
       <c r="H24" s="3">
         <v>40.0</v>
       </c>
@@ -5753,7 +5797,9 @@
       <c r="F25" s="3">
         <v>400.0</v>
       </c>
-      <c r="G25" s="3"/>
+      <c r="G25" s="3">
+        <v>100.0</v>
+      </c>
       <c r="H25" s="3">
         <v>40.0</v>
       </c>
@@ -5790,7 +5836,9 @@
       <c r="F26" s="3">
         <v>400.0</v>
       </c>
-      <c r="G26" s="3"/>
+      <c r="G26" s="3">
+        <v>100.0</v>
+      </c>
       <c r="H26" s="3">
         <v>40.0</v>
       </c>
@@ -5827,7 +5875,9 @@
       <c r="F27" s="3">
         <v>400.0</v>
       </c>
-      <c r="G27" s="3"/>
+      <c r="G27" s="3">
+        <v>100.0</v>
+      </c>
       <c r="H27" s="3">
         <v>40.0</v>
       </c>
@@ -5864,7 +5914,9 @@
       <c r="F28" s="3">
         <v>400.0</v>
       </c>
-      <c r="G28" s="3"/>
+      <c r="G28" s="3">
+        <v>100.0</v>
+      </c>
       <c r="H28" s="3">
         <v>40.0</v>
       </c>
@@ -5901,7 +5953,9 @@
       <c r="F29" s="3">
         <v>400.0</v>
       </c>
-      <c r="G29" s="3"/>
+      <c r="G29" s="3">
+        <v>100.0</v>
+      </c>
       <c r="H29" s="3">
         <v>40.0</v>
       </c>
@@ -5938,7 +5992,9 @@
       <c r="F30" s="3">
         <v>400.0</v>
       </c>
-      <c r="G30" s="3"/>
+      <c r="G30" s="3">
+        <v>100.0</v>
+      </c>
       <c r="H30" s="3">
         <v>40.0</v>
       </c>
@@ -5975,7 +6031,9 @@
       <c r="F31" s="3">
         <v>400.0</v>
       </c>
-      <c r="G31" s="3"/>
+      <c r="G31" s="3">
+        <v>100.0</v>
+      </c>
       <c r="H31" s="3">
         <v>40.0</v>
       </c>
@@ -6012,7 +6070,9 @@
       <c r="F32" s="3">
         <v>400.0</v>
       </c>
-      <c r="G32" s="3"/>
+      <c r="G32" s="3">
+        <v>100.0</v>
+      </c>
       <c r="H32" s="3">
         <v>40.0</v>
       </c>
@@ -6049,7 +6109,9 @@
       <c r="F33" s="3">
         <v>400.0</v>
       </c>
-      <c r="G33" s="3"/>
+      <c r="G33" s="3">
+        <v>100.0</v>
+      </c>
       <c r="H33" s="3">
         <v>40.0</v>
       </c>
@@ -6086,7 +6148,9 @@
       <c r="F34" s="3">
         <v>400.0</v>
       </c>
-      <c r="G34" s="3"/>
+      <c r="G34" s="3">
+        <v>100.0</v>
+      </c>
       <c r="H34" s="3">
         <v>40.0</v>
       </c>
@@ -6123,7 +6187,9 @@
       <c r="F35" s="3">
         <v>400.0</v>
       </c>
-      <c r="G35" s="3"/>
+      <c r="G35" s="3">
+        <v>100.0</v>
+      </c>
       <c r="H35" s="3">
         <v>40.0</v>
       </c>
@@ -6160,7 +6226,9 @@
       <c r="F36" s="3">
         <v>400.0</v>
       </c>
-      <c r="G36" s="3"/>
+      <c r="G36" s="3">
+        <v>100.0</v>
+      </c>
       <c r="H36" s="3">
         <v>40.0</v>
       </c>
@@ -6197,7 +6265,9 @@
       <c r="F37" s="3">
         <v>400.0</v>
       </c>
-      <c r="G37" s="3"/>
+      <c r="G37" s="3">
+        <v>100.0</v>
+      </c>
       <c r="H37" s="3">
         <v>40.0</v>
       </c>
@@ -6234,7 +6304,9 @@
       <c r="F38" s="3">
         <v>400.0</v>
       </c>
-      <c r="G38" s="3"/>
+      <c r="G38" s="3">
+        <v>100.0</v>
+      </c>
       <c r="H38" s="3">
         <v>40.0</v>
       </c>
@@ -6271,7 +6343,9 @@
       <c r="F39" s="3">
         <v>400.0</v>
       </c>
-      <c r="G39" s="3"/>
+      <c r="G39" s="3">
+        <v>100.0</v>
+      </c>
       <c r="H39" s="3">
         <v>40.0</v>
       </c>
@@ -6308,7 +6382,9 @@
       <c r="F40" s="3">
         <v>400.0</v>
       </c>
-      <c r="G40" s="3"/>
+      <c r="G40" s="3">
+        <v>100.0</v>
+      </c>
       <c r="H40" s="3">
         <v>40.0</v>
       </c>
@@ -6345,7 +6421,9 @@
       <c r="F41" s="3">
         <v>400.0</v>
       </c>
-      <c r="G41" s="3"/>
+      <c r="G41" s="3">
+        <v>100.0</v>
+      </c>
       <c r="H41" s="3">
         <v>40.0</v>
       </c>
@@ -6382,7 +6460,9 @@
       <c r="F42" s="3">
         <v>0.0</v>
       </c>
-      <c r="G42" s="3"/>
+      <c r="G42" s="3">
+        <v>100.0</v>
+      </c>
       <c r="H42" s="3">
         <v>40.0</v>
       </c>
@@ -6419,7 +6499,9 @@
       <c r="F43" s="3">
         <v>0.0</v>
       </c>
-      <c r="G43" s="3"/>
+      <c r="G43" s="3">
+        <v>100.0</v>
+      </c>
       <c r="H43" s="3">
         <v>40.0</v>
       </c>
@@ -6456,7 +6538,9 @@
       <c r="F44" s="3">
         <v>0.0</v>
       </c>
-      <c r="G44" s="3"/>
+      <c r="G44" s="3">
+        <v>100.0</v>
+      </c>
       <c r="H44" s="3">
         <v>40.0</v>
       </c>
@@ -6493,7 +6577,9 @@
       <c r="F45" s="3">
         <v>0.0</v>
       </c>
-      <c r="G45" s="3"/>
+      <c r="G45" s="3">
+        <v>100.0</v>
+      </c>
       <c r="H45" s="3">
         <v>40.0</v>
       </c>
@@ -6530,7 +6616,9 @@
       <c r="F46" s="3">
         <v>0.0</v>
       </c>
-      <c r="G46" s="3"/>
+      <c r="G46" s="3">
+        <v>100.0</v>
+      </c>
       <c r="H46" s="3">
         <v>40.0</v>
       </c>
@@ -6567,7 +6655,9 @@
       <c r="F47" s="3">
         <v>0.0</v>
       </c>
-      <c r="G47" s="3"/>
+      <c r="G47" s="3">
+        <v>100.0</v>
+      </c>
       <c r="H47" s="3">
         <v>40.0</v>
       </c>
@@ -6604,7 +6694,9 @@
       <c r="F48" s="3">
         <v>0.0</v>
       </c>
-      <c r="G48" s="3"/>
+      <c r="G48" s="3">
+        <v>100.0</v>
+      </c>
       <c r="H48" s="3">
         <v>40.0</v>
       </c>
@@ -6641,7 +6733,9 @@
       <c r="F49" s="3">
         <v>0.6235014079</v>
       </c>
-      <c r="G49" s="3"/>
+      <c r="G49" s="3">
+        <v>100.0</v>
+      </c>
       <c r="H49" s="3">
         <v>40.0</v>
       </c>
@@ -6678,7 +6772,9 @@
       <c r="F50" s="3">
         <v>32.5488345822</v>
       </c>
-      <c r="G50" s="3"/>
+      <c r="G50" s="3">
+        <v>100.0</v>
+      </c>
       <c r="H50" s="3">
         <v>40.0</v>
       </c>
@@ -6715,7 +6811,9 @@
       <c r="F51" s="3">
         <v>64.4741677564</v>
       </c>
-      <c r="G51" s="3"/>
+      <c r="G51" s="3">
+        <v>100.0</v>
+      </c>
       <c r="H51" s="3">
         <v>40.0</v>
       </c>
@@ -6752,7 +6850,9 @@
       <c r="F52" s="3">
         <v>149.8739824262</v>
       </c>
-      <c r="G52" s="3"/>
+      <c r="G52" s="3">
+        <v>100.0</v>
+      </c>
       <c r="H52" s="3">
         <v>40.0</v>
       </c>
@@ -6789,7 +6889,9 @@
       <c r="F53">
         <v>96.3995009307</v>
       </c>
-      <c r="G53"/>
+      <c r="G53">
+        <v>100.0</v>
+      </c>
       <c r="H53">
         <v>40.0</v>
       </c>
@@ -6826,7 +6928,9 @@
       <c r="F54">
         <v>192.7313415034</v>
       </c>
-      <c r="G54"/>
+      <c r="G54">
+        <v>100.0</v>
+      </c>
       <c r="H54">
         <v>40.0</v>
       </c>
@@ -6863,7 +6967,9 @@
       <c r="F55">
         <v>128.324834105</v>
       </c>
-      <c r="G55"/>
+      <c r="G55">
+        <v>100.0</v>
+      </c>
       <c r="H55">
         <v>40.0</v>
       </c>
@@ -6900,7 +7006,9 @@
       <c r="F56">
         <v>235.5887005806</v>
       </c>
-      <c r="G56"/>
+      <c r="G56">
+        <v>100.0</v>
+      </c>
       <c r="H56">
         <v>40.0</v>
       </c>
@@ -6937,7 +7045,9 @@
       <c r="F57">
         <v>278.4460596578</v>
       </c>
-      <c r="G57"/>
+      <c r="G57">
+        <v>100.0</v>
+      </c>
       <c r="H57">
         <v>40.0</v>
       </c>
@@ -6974,7 +7084,9 @@
       <c r="F58">
         <v>321.303418735</v>
       </c>
-      <c r="G58"/>
+      <c r="G58">
+        <v>100.0</v>
+      </c>
       <c r="H58">
         <v>40.0</v>
       </c>
@@ -7011,7 +7123,9 @@
       <c r="F59">
         <v>364.1607778122</v>
       </c>
-      <c r="G59"/>
+      <c r="G59">
+        <v>100.0</v>
+      </c>
       <c r="H59">
         <v>40.0</v>
       </c>
@@ -9692,14 +9806,14 @@
       <c r="D11" s="3"/>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>mc</t>
+          <t>elastic</t>
         </is>
       </c>
       <c r="F11" s="3">
-        <v>675.0</v>
+        <v>0.0</v>
       </c>
       <c r="G11" s="3">
-        <v>43.0</v>
+        <v>0.0</v>
       </c>
       <c r="H11" s="3"/>
       <c r="I11" s="3">

</xml_diff>

<commit_message>
verification(rs2 joints): the Lorig & Varona rows are posed with friction-only joints; RJ-20 closes at 2.541
UDEC's numbers for RJ-3, RJ-4, RJ-5 and RJ-7 come from the source chapter, whose
joints are friction only; the vendor's file adds 100 kPa of cohesion, which RS2
used. Norm's ruling of 2026-10-02 (Q36 a): the four rows take the chapter's
joints and the vendor's rock; the vendor's-file numbers stay beside as a note.
Re-solved: RJ-3 1.115 (UDEC 1.13, -1.3%, green), RJ-4 1.232 (1.3, -5.2%,
yellow), RJ-5 1.799 (1.7, +5.8%, yellow), RJ-7 1.486 (1.5, -0.9%, green). RJ-20,
whose trial at 2.531 now stands under the contact-cycle rule, closes at 2.541
(UDEC 2.46, +3.3%, yellow) and gains a tag. Figures from the runs' own captures;
page recertified.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/verification/files/rocscience/joints/rj003.xlsx
+++ b/docs/verification/files/rocscience/joints/rj003.xlsx
@@ -4939,9 +4939,7 @@
       <c r="F3" s="3">
         <v>51.9993775139</v>
       </c>
-      <c r="G3" s="3">
-        <v>100.0</v>
-      </c>
+      <c r="G3" s="3"/>
       <c r="H3" s="3">
         <v>40.0</v>
       </c>
@@ -4978,9 +4976,7 @@
       <c r="F4" s="3">
         <v>110.4754655171</v>
       </c>
-      <c r="G4" s="3">
-        <v>100.0</v>
-      </c>
+      <c r="G4" s="3"/>
       <c r="H4" s="3">
         <v>40.0</v>
       </c>
@@ -5017,9 +5013,7 @@
       <c r="F5" s="3">
         <v>140.0</v>
       </c>
-      <c r="G5" s="3">
-        <v>100.0</v>
-      </c>
+      <c r="G5" s="3"/>
       <c r="H5" s="3">
         <v>40.0</v>
       </c>
@@ -5056,9 +5050,7 @@
       <c r="F6" s="3">
         <v>140.0</v>
       </c>
-      <c r="G6" s="3">
-        <v>100.0</v>
-      </c>
+      <c r="G6" s="3"/>
       <c r="H6" s="3">
         <v>40.0</v>
       </c>
@@ -5095,9 +5087,7 @@
       <c r="F7" s="3">
         <v>140.0</v>
       </c>
-      <c r="G7" s="3">
-        <v>100.0</v>
-      </c>
+      <c r="G7" s="3"/>
       <c r="H7" s="3">
         <v>40.0</v>
       </c>
@@ -5134,9 +5124,7 @@
       <c r="F8" s="3">
         <v>140.0</v>
       </c>
-      <c r="G8" s="3">
-        <v>100.0</v>
-      </c>
+      <c r="G8" s="3"/>
       <c r="H8" s="3">
         <v>40.0</v>
       </c>
@@ -5173,9 +5161,7 @@
       <c r="F9" s="3">
         <v>140.0</v>
       </c>
-      <c r="G9" s="3">
-        <v>100.0</v>
-      </c>
+      <c r="G9" s="3"/>
       <c r="H9" s="3">
         <v>40.0</v>
       </c>
@@ -5212,9 +5198,7 @@
       <c r="F10" s="3">
         <v>140.0</v>
       </c>
-      <c r="G10" s="3">
-        <v>100.0</v>
-      </c>
+      <c r="G10" s="3"/>
       <c r="H10" s="3">
         <v>40.0</v>
       </c>
@@ -5251,9 +5235,7 @@
       <c r="F11" s="3">
         <v>140.0</v>
       </c>
-      <c r="G11" s="3">
-        <v>100.0</v>
-      </c>
+      <c r="G11" s="3"/>
       <c r="H11" s="3">
         <v>40.0</v>
       </c>
@@ -5290,9 +5272,7 @@
       <c r="F12" s="3">
         <v>158.3344152734</v>
       </c>
-      <c r="G12" s="3">
-        <v>100.0</v>
-      </c>
+      <c r="G12" s="3"/>
       <c r="H12" s="3">
         <v>40.0</v>
       </c>
@@ -5329,9 +5309,7 @@
       <c r="F13" s="3">
         <v>178.322823806</v>
       </c>
-      <c r="G13" s="3">
-        <v>100.0</v>
-      </c>
+      <c r="G13" s="3"/>
       <c r="H13" s="3">
         <v>40.0</v>
       </c>
@@ -5368,9 +5346,7 @@
       <c r="F14" s="3">
         <v>198.3112323386</v>
       </c>
-      <c r="G14" s="3">
-        <v>100.0</v>
-      </c>
+      <c r="G14" s="3"/>
       <c r="H14" s="3">
         <v>40.0</v>
       </c>
@@ -5407,9 +5383,7 @@
       <c r="F15" s="3">
         <v>218.2996408711</v>
       </c>
-      <c r="G15" s="3">
-        <v>100.0</v>
-      </c>
+      <c r="G15" s="3"/>
       <c r="H15" s="3">
         <v>40.0</v>
       </c>
@@ -5446,9 +5420,7 @@
       <c r="F16" s="3">
         <v>238.2880494037</v>
       </c>
-      <c r="G16" s="3">
-        <v>100.0</v>
-      </c>
+      <c r="G16" s="3"/>
       <c r="H16" s="3">
         <v>40.0</v>
       </c>
@@ -5485,9 +5457,7 @@
       <c r="F17" s="3">
         <v>258.2764579362</v>
       </c>
-      <c r="G17" s="3">
-        <v>100.0</v>
-      </c>
+      <c r="G17" s="3"/>
       <c r="H17" s="3">
         <v>40.0</v>
       </c>
@@ -5524,9 +5494,7 @@
       <c r="F18" s="3">
         <v>278.2648664688</v>
       </c>
-      <c r="G18" s="3">
-        <v>100.0</v>
-      </c>
+      <c r="G18" s="3"/>
       <c r="H18" s="3">
         <v>40.0</v>
       </c>
@@ -5563,9 +5531,7 @@
       <c r="F19" s="3">
         <v>298.2532750014</v>
       </c>
-      <c r="G19" s="3">
-        <v>100.0</v>
-      </c>
+      <c r="G19" s="3"/>
       <c r="H19" s="3">
         <v>40.0</v>
       </c>
@@ -5602,9 +5568,7 @@
       <c r="F20" s="3">
         <v>318.2416835339</v>
       </c>
-      <c r="G20" s="3">
-        <v>100.0</v>
-      </c>
+      <c r="G20" s="3"/>
       <c r="H20" s="3">
         <v>40.0</v>
       </c>
@@ -5641,9 +5605,7 @@
       <c r="F21" s="3">
         <v>338.2300920665</v>
       </c>
-      <c r="G21" s="3">
-        <v>100.0</v>
-      </c>
+      <c r="G21" s="3"/>
       <c r="H21" s="3">
         <v>40.0</v>
       </c>
@@ -5680,9 +5642,7 @@
       <c r="F22" s="3">
         <v>358.2185005991</v>
       </c>
-      <c r="G22" s="3">
-        <v>100.0</v>
-      </c>
+      <c r="G22" s="3"/>
       <c r="H22" s="3">
         <v>40.0</v>
       </c>
@@ -5719,9 +5679,7 @@
       <c r="F23" s="3">
         <v>378.2069091316</v>
       </c>
-      <c r="G23" s="3">
-        <v>100.0</v>
-      </c>
+      <c r="G23" s="3"/>
       <c r="H23" s="3">
         <v>40.0</v>
       </c>
@@ -5758,9 +5716,7 @@
       <c r="F24" s="3">
         <v>398.1953176642</v>
       </c>
-      <c r="G24" s="3">
-        <v>100.0</v>
-      </c>
+      <c r="G24" s="3"/>
       <c r="H24" s="3">
         <v>40.0</v>
       </c>
@@ -5797,9 +5753,7 @@
       <c r="F25" s="3">
         <v>400.0</v>
       </c>
-      <c r="G25" s="3">
-        <v>100.0</v>
-      </c>
+      <c r="G25" s="3"/>
       <c r="H25" s="3">
         <v>40.0</v>
       </c>
@@ -5836,9 +5790,7 @@
       <c r="F26" s="3">
         <v>400.0</v>
       </c>
-      <c r="G26" s="3">
-        <v>100.0</v>
-      </c>
+      <c r="G26" s="3"/>
       <c r="H26" s="3">
         <v>40.0</v>
       </c>
@@ -5875,9 +5827,7 @@
       <c r="F27" s="3">
         <v>400.0</v>
       </c>
-      <c r="G27" s="3">
-        <v>100.0</v>
-      </c>
+      <c r="G27" s="3"/>
       <c r="H27" s="3">
         <v>40.0</v>
       </c>
@@ -5914,9 +5864,7 @@
       <c r="F28" s="3">
         <v>400.0</v>
       </c>
-      <c r="G28" s="3">
-        <v>100.0</v>
-      </c>
+      <c r="G28" s="3"/>
       <c r="H28" s="3">
         <v>40.0</v>
       </c>
@@ -5953,9 +5901,7 @@
       <c r="F29" s="3">
         <v>400.0</v>
       </c>
-      <c r="G29" s="3">
-        <v>100.0</v>
-      </c>
+      <c r="G29" s="3"/>
       <c r="H29" s="3">
         <v>40.0</v>
       </c>
@@ -5992,9 +5938,7 @@
       <c r="F30" s="3">
         <v>400.0</v>
       </c>
-      <c r="G30" s="3">
-        <v>100.0</v>
-      </c>
+      <c r="G30" s="3"/>
       <c r="H30" s="3">
         <v>40.0</v>
       </c>
@@ -6031,9 +5975,7 @@
       <c r="F31" s="3">
         <v>400.0</v>
       </c>
-      <c r="G31" s="3">
-        <v>100.0</v>
-      </c>
+      <c r="G31" s="3"/>
       <c r="H31" s="3">
         <v>40.0</v>
       </c>
@@ -6070,9 +6012,7 @@
       <c r="F32" s="3">
         <v>400.0</v>
       </c>
-      <c r="G32" s="3">
-        <v>100.0</v>
-      </c>
+      <c r="G32" s="3"/>
       <c r="H32" s="3">
         <v>40.0</v>
       </c>
@@ -6109,9 +6049,7 @@
       <c r="F33" s="3">
         <v>400.0</v>
       </c>
-      <c r="G33" s="3">
-        <v>100.0</v>
-      </c>
+      <c r="G33" s="3"/>
       <c r="H33" s="3">
         <v>40.0</v>
       </c>
@@ -6148,9 +6086,7 @@
       <c r="F34" s="3">
         <v>400.0</v>
       </c>
-      <c r="G34" s="3">
-        <v>100.0</v>
-      </c>
+      <c r="G34" s="3"/>
       <c r="H34" s="3">
         <v>40.0</v>
       </c>
@@ -6187,9 +6123,7 @@
       <c r="F35" s="3">
         <v>400.0</v>
       </c>
-      <c r="G35" s="3">
-        <v>100.0</v>
-      </c>
+      <c r="G35" s="3"/>
       <c r="H35" s="3">
         <v>40.0</v>
       </c>
@@ -6226,9 +6160,7 @@
       <c r="F36" s="3">
         <v>400.0</v>
       </c>
-      <c r="G36" s="3">
-        <v>100.0</v>
-      </c>
+      <c r="G36" s="3"/>
       <c r="H36" s="3">
         <v>40.0</v>
       </c>
@@ -6265,9 +6197,7 @@
       <c r="F37" s="3">
         <v>400.0</v>
       </c>
-      <c r="G37" s="3">
-        <v>100.0</v>
-      </c>
+      <c r="G37" s="3"/>
       <c r="H37" s="3">
         <v>40.0</v>
       </c>
@@ -6304,9 +6234,7 @@
       <c r="F38" s="3">
         <v>400.0</v>
       </c>
-      <c r="G38" s="3">
-        <v>100.0</v>
-      </c>
+      <c r="G38" s="3"/>
       <c r="H38" s="3">
         <v>40.0</v>
       </c>
@@ -6343,9 +6271,7 @@
       <c r="F39" s="3">
         <v>400.0</v>
       </c>
-      <c r="G39" s="3">
-        <v>100.0</v>
-      </c>
+      <c r="G39" s="3"/>
       <c r="H39" s="3">
         <v>40.0</v>
       </c>
@@ -6382,9 +6308,7 @@
       <c r="F40" s="3">
         <v>400.0</v>
       </c>
-      <c r="G40" s="3">
-        <v>100.0</v>
-      </c>
+      <c r="G40" s="3"/>
       <c r="H40" s="3">
         <v>40.0</v>
       </c>
@@ -6421,9 +6345,7 @@
       <c r="F41" s="3">
         <v>400.0</v>
       </c>
-      <c r="G41" s="3">
-        <v>100.0</v>
-      </c>
+      <c r="G41" s="3"/>
       <c r="H41" s="3">
         <v>40.0</v>
       </c>
@@ -6460,9 +6382,7 @@
       <c r="F42" s="3">
         <v>0.0</v>
       </c>
-      <c r="G42" s="3">
-        <v>100.0</v>
-      </c>
+      <c r="G42" s="3"/>
       <c r="H42" s="3">
         <v>40.0</v>
       </c>
@@ -6499,9 +6419,7 @@
       <c r="F43" s="3">
         <v>0.0</v>
       </c>
-      <c r="G43" s="3">
-        <v>100.0</v>
-      </c>
+      <c r="G43" s="3"/>
       <c r="H43" s="3">
         <v>40.0</v>
       </c>
@@ -6538,9 +6456,7 @@
       <c r="F44" s="3">
         <v>0.0</v>
       </c>
-      <c r="G44" s="3">
-        <v>100.0</v>
-      </c>
+      <c r="G44" s="3"/>
       <c r="H44" s="3">
         <v>40.0</v>
       </c>
@@ -6577,9 +6493,7 @@
       <c r="F45" s="3">
         <v>0.0</v>
       </c>
-      <c r="G45" s="3">
-        <v>100.0</v>
-      </c>
+      <c r="G45" s="3"/>
       <c r="H45" s="3">
         <v>40.0</v>
       </c>
@@ -6616,9 +6530,7 @@
       <c r="F46" s="3">
         <v>0.0</v>
       </c>
-      <c r="G46" s="3">
-        <v>100.0</v>
-      </c>
+      <c r="G46" s="3"/>
       <c r="H46" s="3">
         <v>40.0</v>
       </c>
@@ -6655,9 +6567,7 @@
       <c r="F47" s="3">
         <v>0.0</v>
       </c>
-      <c r="G47" s="3">
-        <v>100.0</v>
-      </c>
+      <c r="G47" s="3"/>
       <c r="H47" s="3">
         <v>40.0</v>
       </c>
@@ -6694,9 +6604,7 @@
       <c r="F48" s="3">
         <v>0.0</v>
       </c>
-      <c r="G48" s="3">
-        <v>100.0</v>
-      </c>
+      <c r="G48" s="3"/>
       <c r="H48" s="3">
         <v>40.0</v>
       </c>
@@ -6733,9 +6641,7 @@
       <c r="F49" s="3">
         <v>0.6235014079</v>
       </c>
-      <c r="G49" s="3">
-        <v>100.0</v>
-      </c>
+      <c r="G49" s="3"/>
       <c r="H49" s="3">
         <v>40.0</v>
       </c>
@@ -6772,9 +6678,7 @@
       <c r="F50" s="3">
         <v>32.5488345822</v>
       </c>
-      <c r="G50" s="3">
-        <v>100.0</v>
-      </c>
+      <c r="G50" s="3"/>
       <c r="H50" s="3">
         <v>40.0</v>
       </c>
@@ -6811,9 +6715,7 @@
       <c r="F51" s="3">
         <v>64.4741677564</v>
       </c>
-      <c r="G51" s="3">
-        <v>100.0</v>
-      </c>
+      <c r="G51" s="3"/>
       <c r="H51" s="3">
         <v>40.0</v>
       </c>
@@ -6850,9 +6752,7 @@
       <c r="F52" s="3">
         <v>149.8739824262</v>
       </c>
-      <c r="G52" s="3">
-        <v>100.0</v>
-      </c>
+      <c r="G52" s="3"/>
       <c r="H52" s="3">
         <v>40.0</v>
       </c>
@@ -6889,9 +6789,7 @@
       <c r="F53">
         <v>96.3995009307</v>
       </c>
-      <c r="G53">
-        <v>100.0</v>
-      </c>
+      <c r="G53"/>
       <c r="H53">
         <v>40.0</v>
       </c>
@@ -6928,9 +6826,7 @@
       <c r="F54">
         <v>192.7313415034</v>
       </c>
-      <c r="G54">
-        <v>100.0</v>
-      </c>
+      <c r="G54"/>
       <c r="H54">
         <v>40.0</v>
       </c>
@@ -6967,9 +6863,7 @@
       <c r="F55">
         <v>128.324834105</v>
       </c>
-      <c r="G55">
-        <v>100.0</v>
-      </c>
+      <c r="G55"/>
       <c r="H55">
         <v>40.0</v>
       </c>
@@ -7006,9 +6900,7 @@
       <c r="F56">
         <v>235.5887005806</v>
       </c>
-      <c r="G56">
-        <v>100.0</v>
-      </c>
+      <c r="G56"/>
       <c r="H56">
         <v>40.0</v>
       </c>
@@ -7045,9 +6937,7 @@
       <c r="F57">
         <v>278.4460596578</v>
       </c>
-      <c r="G57">
-        <v>100.0</v>
-      </c>
+      <c r="G57"/>
       <c r="H57">
         <v>40.0</v>
       </c>
@@ -7084,9 +6974,7 @@
       <c r="F58">
         <v>321.303418735</v>
       </c>
-      <c r="G58">
-        <v>100.0</v>
-      </c>
+      <c r="G58"/>
       <c r="H58">
         <v>40.0</v>
       </c>
@@ -7123,9 +7011,7 @@
       <c r="F59">
         <v>364.1607778122</v>
       </c>
-      <c r="G59">
-        <v>100.0</v>
-      </c>
+      <c r="G59"/>
       <c r="H59">
         <v>40.0</v>
       </c>

</xml_diff>